<commit_message>
duplicate schema script works
</commit_message>
<xml_diff>
--- a/static/example_sheets_online/eDNA archive sampling.xlsx
+++ b/static/example_sheets_online/eDNA archive sampling.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\glj523\Documents\github repoes\upload_web_app\example_sheets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\glj523\Documents\github repoes\upload_web_app\static\example_sheets_online\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B4DFB46-97DB-4D9C-9B7E-790FCFAA9320}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FC86347-CDF4-4120-BBC8-EF827ABA8E9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{F20BE04D-14A6-4DFA-9322-DA461E992517}"/>
+    <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{F20BE04D-14A6-4DFA-9322-DA461E992517}"/>
   </bookViews>
   <sheets>
     <sheet name="eDNA_Archive_sampling_(20231027" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="ExternalData_1" localSheetId="0" hidden="1">'eDNA_Archive_sampling_(20231027'!$B$1:$Q$6</definedName>
+    <definedName name="ExternalData_1" localSheetId="0" hidden="1">'eDNA_Archive_sampling_(20231027'!$B$1:$Q$4</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="36">
   <si>
     <t>low</t>
   </si>
@@ -55,21 +55,9 @@
     <t>Expected column names and positions:</t>
   </si>
   <si>
-    <t>Expected data type:</t>
-  </si>
-  <si>
     <t>Example of accepted data:</t>
   </si>
   <si>
-    <t>yes</t>
-  </si>
-  <si>
-    <t>text and/or number(s)</t>
-  </si>
-  <si>
-    <t>text</t>
-  </si>
-  <si>
     <t>no</t>
   </si>
   <si>
@@ -127,9 +115,6 @@
     <t>NotesSubmitter</t>
   </si>
   <si>
-    <t>number (decimal allowed)</t>
-  </si>
-  <si>
     <t>LV3005888119</t>
   </si>
   <si>
@@ -167,15 +152,6 @@
   </si>
   <si>
     <t>YYYY-MM-DD or DD-MM-YYYY</t>
-  </si>
-  <si>
-    <t>Required?*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">*Indicates if a cell is allowed to be empty or not. </t>
-  </si>
-  <si>
-    <t>date or free text</t>
   </si>
   <si>
     <t>KU-ID, seperated by semicolon if multiple</t>
@@ -362,8 +338,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{55D4DEA4-CA91-4296-BF11-ADA08522FD65}" name="eDNA_Archive_sampling__20231027_NKL_CAM2204" displayName="eDNA_Archive_sampling__20231027_NKL_CAM2204" ref="B1:Q6" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="B1:Q6" xr:uid="{55D4DEA4-CA91-4296-BF11-ADA08522FD65}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{55D4DEA4-CA91-4296-BF11-ADA08522FD65}" name="eDNA_Archive_sampling__20231027_NKL_CAM2204" displayName="eDNA_Archive_sampling__20231027_NKL_CAM2204" ref="B1:Q4" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="B1:Q4" xr:uid="{55D4DEA4-CA91-4296-BF11-ADA08522FD65}"/>
   <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{A6C9380F-783C-4775-A6B6-D38824DA3359}" uniqueName="1" name="ArchiveSampleID" queryTableFieldId="1" dataDxfId="13"/>
     <tableColumn id="2" xr3:uid="{809C253B-4C6E-4ABA-965D-821AA778382E}" uniqueName="2" name="PositionInRack" queryTableFieldId="2" dataDxfId="12"/>
@@ -387,9 +363,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -427,7 +403,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -533,7 +509,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -675,7 +651,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -683,7 +659,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92B8DB45-AD95-4AEF-BE44-A884078F1D25}">
-  <dimension ref="A1:Q9"/>
+  <dimension ref="A1:Q4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="41.88671875" bestFit="1" customWidth="1"/>
@@ -706,221 +682,130 @@
         <v>1</v>
       </c>
       <c r="B1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" t="s">
         <v>10</v>
       </c>
-      <c r="C1" t="s">
+      <c r="G1" t="s">
         <v>11</v>
       </c>
-      <c r="D1" t="s">
+      <c r="H1" t="s">
         <v>12</v>
       </c>
-      <c r="E1" t="s">
+      <c r="I1" t="s">
         <v>13</v>
       </c>
-      <c r="F1" t="s">
+      <c r="J1" t="s">
         <v>14</v>
       </c>
-      <c r="G1" t="s">
+      <c r="K1" t="s">
         <v>15</v>
       </c>
-      <c r="H1" t="s">
+      <c r="L1" t="s">
         <v>16</v>
       </c>
-      <c r="I1" t="s">
+      <c r="M1" t="s">
         <v>17</v>
       </c>
-      <c r="J1" t="s">
+      <c r="N1" t="s">
         <v>18</v>
       </c>
-      <c r="K1" t="s">
+      <c r="O1" t="s">
         <v>19</v>
       </c>
-      <c r="L1" t="s">
+      <c r="P1" t="s">
         <v>20</v>
       </c>
-      <c r="M1" t="s">
+      <c r="Q1" t="s">
         <v>21</v>
       </c>
-      <c r="N1" t="s">
-        <v>22</v>
-      </c>
-      <c r="O1" t="s">
-        <v>23</v>
-      </c>
-      <c r="P1" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>25</v>
-      </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G2">
+        <v>100.5</v>
+      </c>
+      <c r="I2" t="s">
+        <v>0</v>
+      </c>
+      <c r="J2" t="s">
+        <v>3</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="L2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
+      <c r="O2" t="s">
+        <v>29</v>
+      </c>
+      <c r="P2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G2" t="s">
-        <v>26</v>
-      </c>
-      <c r="H2" t="s">
-        <v>5</v>
-      </c>
-      <c r="I2" t="s">
-        <v>6</v>
-      </c>
-      <c r="J2" t="s">
-        <v>6</v>
-      </c>
-      <c r="K2" t="s">
-        <v>5</v>
-      </c>
-      <c r="L2" t="s">
-        <v>5</v>
-      </c>
-      <c r="M2" t="s">
-        <v>5</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="O2" t="s">
-        <v>5</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>42</v>
-      </c>
       <c r="Q2" t="s">
-        <v>5</v>
+        <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D3" t="s">
-        <v>29</v>
-      </c>
-      <c r="E3" t="s">
-        <v>30</v>
-      </c>
-      <c r="F3" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="G3">
-        <v>100.5</v>
-      </c>
-      <c r="I3" t="s">
-        <v>0</v>
-      </c>
-      <c r="J3" t="s">
-        <v>7</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>8</v>
-      </c>
+      <c r="K3" s="1"/>
       <c r="L3" t="s">
         <v>32</v>
       </c>
       <c r="M3" t="s">
-        <v>33</v>
-      </c>
-      <c r="N3" s="2" t="s">
-        <v>9</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="N3" s="1"/>
       <c r="O3" t="s">
-        <v>34</v>
-      </c>
-      <c r="P3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q3" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" t="s">
-        <v>4</v>
-      </c>
-      <c r="D4" t="s">
-        <v>4</v>
-      </c>
-      <c r="E4" t="s">
-        <v>4</v>
-      </c>
-      <c r="F4" t="s">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="K4" s="1"/>
-      <c r="N4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="O4" t="s">
-        <v>4</v>
+      <c r="N4" t="s">
+        <v>34</v>
       </c>
       <c r="P4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K5" s="1"/>
-      <c r="L5" t="s">
-        <v>37</v>
-      </c>
-      <c r="M5" t="s">
-        <v>43</v>
-      </c>
-      <c r="N5" s="1"/>
-      <c r="O5" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>38</v>
-      </c>
-      <c r="K6" s="1"/>
-      <c r="N6" t="s">
-        <v>39</v>
-      </c>
-      <c r="P6" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="K7" s="1"/>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>